<commit_message>
Update the site contact details to the current studio phone, email, and address.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/content/website-copy.xlsx
+++ b/content/website-copy.xlsx
@@ -95,7 +95,7 @@
     <t>Top bar — email label</t>
   </si>
   <si>
-    <t>hello@countyhalldance.co.uk</t>
+    <t>info@countyhalldancecentre.com</t>
   </si>
   <si>
     <t>global.utilitybar.findus.label</t>
@@ -113,7 +113,7 @@
     <t>Top bar — phone label</t>
   </si>
   <si>
-    <t>+44 20 7946 0958</t>
+    <t>+44 7728 617531</t>
   </si>
   <si>
     <t>global.utilitybar.social.facebook.label</t>
@@ -644,7 +644,7 @@
     <t>Footer — contact address line 1</t>
   </si>
   <si>
-    <t>County Hall Dance Studio</t>
+    <t>2nd Floor, County Hall Main Entrance</t>
   </si>
   <si>
     <t>global.footer.contact.address.1</t>
@@ -662,7 +662,7 @@
     <t>Footer — contact address line 3</t>
   </si>
   <si>
-    <t>London SE1 7GP</t>
+    <t>London SE1 7PB</t>
   </si>
   <si>
     <t>global.footer.contact.email</t>
@@ -5958,16 +5958,16 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
@@ -6381,7 +6381,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -14366,6 +14366,6 @@
     <mergeCell ref="A749:C749"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>